<commit_message>
added novel natives to preop session
added new session type, 'preop', separate from 'familiarization,' 'training', and 'test'

for stimulus schematic, go to:
https://docs.google.com/presentation/d/1RF64AF8fRELeEpCeYnjbzqEtENcHat-QyYaIHkaJMMg/edit#slide=id.gc899d3adf8_0_0
</commit_message>
<xml_diff>
--- a/stim/stim_group_lists_familiarization.xlsx
+++ b/stim/stim_group_lists_familiarization.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24701"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\speechres\Task_SpeechMotorSequenceLearning\stim\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amsme\OneDrive\Documents\code\matlab\Task_SpeechMotorSequenceLearning\stim\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C7AE5AE-41C2-49C7-9481-C6C85B559357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{779FD5A7-FF40-4CBB-A984-7B3800407086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1860" yWindow="1860" windowWidth="21600" windowHeight="11385" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,9 +27,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="13">
   <si>
-    <t>native</t>
-  </si>
-  <si>
     <t>group1</t>
   </si>
   <si>
@@ -64,6 +61,9 @@
   </si>
   <si>
     <t>non-native novel</t>
+  </si>
+  <si>
+    <t>native novel</t>
   </si>
 </sst>
 </file>
@@ -436,34 +436,34 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
@@ -489,7 +489,7 @@
         <v>21</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I2" s="1">
         <v>3</v>
@@ -521,7 +521,7 @@
         <v>15</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I3" s="1">
         <v>2</v>
@@ -553,7 +553,7 @@
         <v>22</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I4" s="1">
         <v>3</v>
@@ -585,7 +585,7 @@
         <v>24</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I5" s="1">
         <v>3</v>
@@ -617,7 +617,7 @@
         <v>23</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I6" s="1">
         <v>3</v>
@@ -649,7 +649,7 @@
         <v>16</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I7" s="1">
         <v>2</v>
@@ -681,7 +681,7 @@
         <v>23</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I8" s="1">
         <v>3</v>
@@ -713,7 +713,7 @@
         <v>21</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I9" s="1">
         <v>3</v>
@@ -745,7 +745,7 @@
         <v>17</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I10" s="1">
         <v>2</v>
@@ -777,7 +777,7 @@
         <v>22</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I11" s="1">
         <v>3</v>
@@ -809,7 +809,7 @@
         <v>18</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I12" s="1">
         <v>2</v>
@@ -841,7 +841,7 @@
         <v>24</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I13" s="1">
         <v>3</v>

</xml_diff>

<commit_message>
switched KFAT out out for TFED in learning-familiarization
KFAT overlapped with KFUB in a test phase trained/novel set, so KFAT was giving a little unintentional training
</commit_message>
<xml_diff>
--- a/stim/stim_group_lists_familiarization.xlsx
+++ b/stim/stim_group_lists_familiarization.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24701"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amsme\OneDrive\Documents\code\matlab\Task_SpeechMotorSequenceLearning\stim\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\docs\code\Task_SpeechMotorSequenceLearning\stim\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{779FD5A7-FF40-4CBB-A984-7B3800407086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE5A82A4-138D-4A90-9A33-9BD57C7A9CF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -98,12 +98,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -128,9 +127,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -168,7 +167,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -274,7 +273,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -416,7 +415,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -427,15 +426,15 @@
   <dimension ref="A1:J49"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" style="4"/>
+    <col min="1" max="1" width="11.5703125" style="3"/>
     <col min="2" max="7" width="11.5703125" style="1"/>
     <col min="8" max="8" width="19.5703125" customWidth="1"/>
     <col min="9" max="9" width="8.28515625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="8.28515625" style="3" customWidth="1"/>
+    <col min="10" max="10" width="8.28515625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -467,28 +466,28 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="4">
-        <v>21</v>
-      </c>
-      <c r="B2" s="4">
-        <v>21</v>
-      </c>
-      <c r="C2" s="4">
-        <v>21</v>
-      </c>
-      <c r="D2" s="4">
-        <v>21</v>
-      </c>
-      <c r="E2" s="4">
-        <v>21</v>
-      </c>
-      <c r="F2" s="4">
-        <v>21</v>
-      </c>
-      <c r="G2" s="4">
-        <v>21</v>
-      </c>
-      <c r="H2" s="2" t="s">
+      <c r="A2" s="3">
+        <v>21</v>
+      </c>
+      <c r="B2" s="3">
+        <v>21</v>
+      </c>
+      <c r="C2" s="3">
+        <v>21</v>
+      </c>
+      <c r="D2" s="3">
+        <v>21</v>
+      </c>
+      <c r="E2" s="3">
+        <v>21</v>
+      </c>
+      <c r="F2" s="3">
+        <v>21</v>
+      </c>
+      <c r="G2" s="3">
+        <v>21</v>
+      </c>
+      <c r="H2" t="s">
         <v>12</v>
       </c>
       <c r="I2" s="1">
@@ -499,28 +498,28 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="4">
+      <c r="A3" s="3">
         <v>15</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="3">
         <v>15</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="3">
         <v>15</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="3">
         <v>15</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="3">
         <v>15</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="3">
         <v>15</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="3">
         <v>15</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" t="s">
         <v>11</v>
       </c>
       <c r="I3" s="1">
@@ -531,28 +530,28 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="4">
-        <v>22</v>
-      </c>
-      <c r="B4" s="4">
-        <v>22</v>
-      </c>
-      <c r="C4" s="4">
-        <v>22</v>
-      </c>
-      <c r="D4" s="4">
-        <v>22</v>
-      </c>
-      <c r="E4" s="4">
-        <v>22</v>
-      </c>
-      <c r="F4" s="4">
-        <v>22</v>
-      </c>
-      <c r="G4" s="4">
-        <v>22</v>
-      </c>
-      <c r="H4" s="2" t="s">
+      <c r="A4" s="3">
+        <v>22</v>
+      </c>
+      <c r="B4" s="3">
+        <v>22</v>
+      </c>
+      <c r="C4" s="3">
+        <v>22</v>
+      </c>
+      <c r="D4" s="3">
+        <v>22</v>
+      </c>
+      <c r="E4" s="3">
+        <v>22</v>
+      </c>
+      <c r="F4" s="3">
+        <v>22</v>
+      </c>
+      <c r="G4" s="3">
+        <v>22</v>
+      </c>
+      <c r="H4" t="s">
         <v>12</v>
       </c>
       <c r="I4" s="1">
@@ -563,28 +562,28 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="4">
-        <v>24</v>
-      </c>
-      <c r="B5" s="4">
-        <v>24</v>
-      </c>
-      <c r="C5" s="4">
-        <v>24</v>
-      </c>
-      <c r="D5" s="4">
-        <v>24</v>
-      </c>
-      <c r="E5" s="4">
-        <v>24</v>
-      </c>
-      <c r="F5" s="4">
-        <v>24</v>
-      </c>
-      <c r="G5" s="4">
-        <v>24</v>
-      </c>
-      <c r="H5" s="2" t="s">
+      <c r="A5" s="3">
+        <v>24</v>
+      </c>
+      <c r="B5" s="3">
+        <v>24</v>
+      </c>
+      <c r="C5" s="3">
+        <v>24</v>
+      </c>
+      <c r="D5" s="3">
+        <v>24</v>
+      </c>
+      <c r="E5" s="3">
+        <v>24</v>
+      </c>
+      <c r="F5" s="3">
+        <v>24</v>
+      </c>
+      <c r="G5" s="3">
+        <v>24</v>
+      </c>
+      <c r="H5" t="s">
         <v>8</v>
       </c>
       <c r="I5" s="1">
@@ -595,28 +594,28 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="4">
-        <v>23</v>
-      </c>
-      <c r="B6" s="4">
-        <v>23</v>
-      </c>
-      <c r="C6" s="4">
-        <v>23</v>
-      </c>
-      <c r="D6" s="4">
-        <v>23</v>
-      </c>
-      <c r="E6" s="4">
-        <v>23</v>
-      </c>
-      <c r="F6" s="4">
-        <v>23</v>
-      </c>
-      <c r="G6" s="4">
-        <v>23</v>
-      </c>
-      <c r="H6" s="2" t="s">
+      <c r="A6" s="3">
+        <v>23</v>
+      </c>
+      <c r="B6" s="3">
+        <v>23</v>
+      </c>
+      <c r="C6" s="3">
+        <v>23</v>
+      </c>
+      <c r="D6" s="3">
+        <v>23</v>
+      </c>
+      <c r="E6" s="3">
+        <v>23</v>
+      </c>
+      <c r="F6" s="3">
+        <v>23</v>
+      </c>
+      <c r="G6" s="3">
+        <v>23</v>
+      </c>
+      <c r="H6" t="s">
         <v>8</v>
       </c>
       <c r="I6" s="1">
@@ -627,28 +626,28 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="4">
-        <v>16</v>
-      </c>
-      <c r="B7" s="4">
-        <v>16</v>
-      </c>
-      <c r="C7" s="4">
-        <v>16</v>
-      </c>
-      <c r="D7" s="4">
-        <v>16</v>
-      </c>
-      <c r="E7" s="4">
-        <v>16</v>
-      </c>
-      <c r="F7" s="4">
-        <v>16</v>
-      </c>
-      <c r="G7" s="4">
-        <v>16</v>
-      </c>
-      <c r="H7" s="2" t="s">
+      <c r="A7" s="3">
+        <v>75</v>
+      </c>
+      <c r="B7" s="3">
+        <v>75</v>
+      </c>
+      <c r="C7" s="3">
+        <v>75</v>
+      </c>
+      <c r="D7" s="3">
+        <v>75</v>
+      </c>
+      <c r="E7" s="3">
+        <v>75</v>
+      </c>
+      <c r="F7" s="3">
+        <v>75</v>
+      </c>
+      <c r="G7" s="3">
+        <v>75</v>
+      </c>
+      <c r="H7" t="s">
         <v>11</v>
       </c>
       <c r="I7" s="1">
@@ -659,28 +658,28 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="4">
-        <v>23</v>
-      </c>
-      <c r="B8" s="4">
-        <v>23</v>
-      </c>
-      <c r="C8" s="4">
-        <v>23</v>
-      </c>
-      <c r="D8" s="4">
-        <v>23</v>
-      </c>
-      <c r="E8" s="4">
-        <v>23</v>
-      </c>
-      <c r="F8" s="4">
-        <v>23</v>
-      </c>
-      <c r="G8" s="4">
-        <v>23</v>
-      </c>
-      <c r="H8" s="2" t="s">
+      <c r="A8" s="3">
+        <v>23</v>
+      </c>
+      <c r="B8" s="3">
+        <v>23</v>
+      </c>
+      <c r="C8" s="3">
+        <v>23</v>
+      </c>
+      <c r="D8" s="3">
+        <v>23</v>
+      </c>
+      <c r="E8" s="3">
+        <v>23</v>
+      </c>
+      <c r="F8" s="3">
+        <v>23</v>
+      </c>
+      <c r="G8" s="3">
+        <v>23</v>
+      </c>
+      <c r="H8" t="s">
         <v>12</v>
       </c>
       <c r="I8" s="1">
@@ -691,28 +690,28 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="4">
-        <v>21</v>
-      </c>
-      <c r="B9" s="4">
-        <v>21</v>
-      </c>
-      <c r="C9" s="4">
-        <v>21</v>
-      </c>
-      <c r="D9" s="4">
-        <v>21</v>
-      </c>
-      <c r="E9" s="4">
-        <v>21</v>
-      </c>
-      <c r="F9" s="4">
-        <v>21</v>
-      </c>
-      <c r="G9" s="4">
-        <v>21</v>
-      </c>
-      <c r="H9" s="2" t="s">
+      <c r="A9" s="3">
+        <v>21</v>
+      </c>
+      <c r="B9" s="3">
+        <v>21</v>
+      </c>
+      <c r="C9" s="3">
+        <v>21</v>
+      </c>
+      <c r="D9" s="3">
+        <v>21</v>
+      </c>
+      <c r="E9" s="3">
+        <v>21</v>
+      </c>
+      <c r="F9" s="3">
+        <v>21</v>
+      </c>
+      <c r="G9" s="3">
+        <v>21</v>
+      </c>
+      <c r="H9" t="s">
         <v>8</v>
       </c>
       <c r="I9" s="1">
@@ -723,28 +722,28 @@
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="4">
+      <c r="A10" s="3">
         <v>17</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="3">
         <v>17</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="3">
         <v>17</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="3">
         <v>17</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="3">
         <v>17</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="3">
         <v>17</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="3">
         <v>17</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" t="s">
         <v>11</v>
       </c>
       <c r="I10" s="1">
@@ -755,28 +754,28 @@
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="4">
-        <v>22</v>
-      </c>
-      <c r="B11" s="4">
-        <v>22</v>
-      </c>
-      <c r="C11" s="4">
-        <v>22</v>
-      </c>
-      <c r="D11" s="4">
-        <v>22</v>
-      </c>
-      <c r="E11" s="4">
-        <v>22</v>
-      </c>
-      <c r="F11" s="4">
-        <v>22</v>
-      </c>
-      <c r="G11" s="4">
-        <v>22</v>
-      </c>
-      <c r="H11" s="2" t="s">
+      <c r="A11" s="3">
+        <v>22</v>
+      </c>
+      <c r="B11" s="3">
+        <v>22</v>
+      </c>
+      <c r="C11" s="3">
+        <v>22</v>
+      </c>
+      <c r="D11" s="3">
+        <v>22</v>
+      </c>
+      <c r="E11" s="3">
+        <v>22</v>
+      </c>
+      <c r="F11" s="3">
+        <v>22</v>
+      </c>
+      <c r="G11" s="3">
+        <v>22</v>
+      </c>
+      <c r="H11" t="s">
         <v>8</v>
       </c>
       <c r="I11" s="1">
@@ -787,28 +786,28 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="4">
+      <c r="A12" s="3">
         <v>18</v>
       </c>
-      <c r="B12" s="4">
+      <c r="B12" s="3">
         <v>18</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C12" s="3">
         <v>18</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12" s="3">
         <v>18</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="3">
         <v>18</v>
       </c>
-      <c r="F12" s="4">
+      <c r="F12" s="3">
         <v>18</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="3">
         <v>18</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H12" t="s">
         <v>11</v>
       </c>
       <c r="I12" s="1">
@@ -819,28 +818,28 @@
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="4">
-        <v>24</v>
-      </c>
-      <c r="B13" s="4">
-        <v>24</v>
-      </c>
-      <c r="C13" s="4">
-        <v>24</v>
-      </c>
-      <c r="D13" s="4">
-        <v>24</v>
-      </c>
-      <c r="E13" s="4">
-        <v>24</v>
-      </c>
-      <c r="F13" s="4">
-        <v>24</v>
-      </c>
-      <c r="G13" s="4">
-        <v>24</v>
-      </c>
-      <c r="H13" s="2" t="s">
+      <c r="A13" s="3">
+        <v>24</v>
+      </c>
+      <c r="B13" s="3">
+        <v>24</v>
+      </c>
+      <c r="C13" s="3">
+        <v>24</v>
+      </c>
+      <c r="D13" s="3">
+        <v>24</v>
+      </c>
+      <c r="E13" s="3">
+        <v>24</v>
+      </c>
+      <c r="F13" s="3">
+        <v>24</v>
+      </c>
+      <c r="G13" s="3">
+        <v>24</v>
+      </c>
+      <c r="H13" t="s">
         <v>12</v>
       </c>
       <c r="I13" s="1">
@@ -850,109 +849,37 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="H14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="H15" s="2"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="H16" s="2"/>
-    </row>
-    <row r="17" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H17" s="2"/>
-    </row>
-    <row r="18" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H18" s="2"/>
-    </row>
-    <row r="19" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H19" s="2"/>
-    </row>
-    <row r="20" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H20" s="2"/>
-    </row>
-    <row r="21" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H21" s="2"/>
-    </row>
-    <row r="22" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H22" s="2"/>
-    </row>
-    <row r="23" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H23" s="2"/>
-    </row>
-    <row r="24" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H24" s="2"/>
-    </row>
-    <row r="25" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H25" s="2"/>
-    </row>
-    <row r="26" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H26" s="2"/>
-    </row>
-    <row r="27" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H27" s="2"/>
-    </row>
-    <row r="28" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H28" s="2"/>
-    </row>
-    <row r="29" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H29" s="2"/>
-    </row>
-    <row r="30" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H30" s="2"/>
-    </row>
-    <row r="31" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H31" s="2"/>
-    </row>
-    <row r="32" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H32" s="2"/>
-    </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="H33" s="2"/>
-    </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="H34" s="2"/>
-    </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="H35" s="2"/>
-    </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="H36" s="2"/>
-    </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="H37" s="2"/>
-    </row>
-    <row r="46" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B46" s="4"/>
-      <c r="C46" s="4"/>
-      <c r="D46" s="4"/>
-      <c r="E46" s="4"/>
-      <c r="F46" s="4"/>
-      <c r="G46" s="4"/>
-    </row>
-    <row r="47" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B47" s="4"/>
-      <c r="C47" s="4"/>
-      <c r="D47" s="4"/>
-      <c r="E47" s="4"/>
-      <c r="F47" s="4"/>
-      <c r="G47" s="4"/>
-    </row>
-    <row r="48" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B48" s="4"/>
-      <c r="C48" s="4"/>
-      <c r="D48" s="4"/>
-      <c r="E48" s="4"/>
-      <c r="F48" s="4"/>
-      <c r="G48" s="4"/>
+    <row r="46" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B46" s="3"/>
+      <c r="C46" s="3"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+    </row>
+    <row r="47" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B47" s="3"/>
+      <c r="C47" s="3"/>
+      <c r="D47" s="3"/>
+      <c r="E47" s="3"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+    </row>
+    <row r="48" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B48" s="3"/>
+      <c r="C48" s="3"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
     </row>
     <row r="49" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B49" s="4"/>
-      <c r="C49" s="4"/>
-      <c r="D49" s="4"/>
-      <c r="E49" s="4"/>
-      <c r="F49" s="4"/>
-      <c r="G49" s="4"/>
+      <c r="B49" s="3"/>
+      <c r="C49" s="3"/>
+      <c r="D49" s="3"/>
+      <c r="E49" s="3"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>

</xml_diff>